<commit_message>
Actualizar datos 2026 (2026-04-09)
</commit_message>
<xml_diff>
--- a/data/asistencia/Guerreros 2026.xlsx
+++ b/data/asistencia/Guerreros 2026.xlsx
@@ -118,7 +118,7 @@
     <t>Palco</t>
   </si>
   <si>
-    <t>70.05%</t>
+    <t>75.00%</t>
   </si>
   <si>
     <t>Zona del Recuerdo</t>
@@ -127,7 +127,7 @@
     <t>TOTALES</t>
   </si>
   <si>
-    <t>4.95%</t>
+    <t>5.18%</t>
   </si>
 </sst>
 </file>
@@ -1083,7 +1083,7 @@
         <v>23</v>
       </c>
       <c r="I13" s="7">
-        <v>254</v>
+        <v>272</v>
       </c>
       <c r="J13" s="7" t="s">
         <v>23</v>
@@ -1107,10 +1107,10 @@
         <v>364</v>
       </c>
       <c r="Q13" s="7">
-        <v>255</v>
+        <v>273</v>
       </c>
       <c r="R13" s="7">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="S13" s="8" t="s">
         <v>35</v>

</xml_diff>